<commit_message>
Update Candle Pattern - Detect all tf
</commit_message>
<xml_diff>
--- a/Experts/Anhnt/Document/MQL5 Note/2026 0731 SettingMarket.xlsx
+++ b/Experts/Anhnt/Document/MQL5 Note/2026 0731 SettingMarket.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\AppData\Roaming\MetaQuotes\Terminal\D0E8209F77C8CF37AD8BF550E51FF075\MQL5\Experts\Anhnt\Document\MQL5 Note\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511A14C6-3E89-48E3-BA5F-F358489D111D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89884ECE-1ACE-432F-8551-52E8EB294E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F58B3433-660C-425C-BE04-949B5E51AFEB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
   <si>
     <t>SETTING_MARKER_BASE_X_GAP</t>
   </si>
@@ -491,7 +491,7 @@
     <col min="3" max="3" width="7.33203125" customWidth="1"/>
     <col min="4" max="4" width="27" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="37.21875" customWidth="1"/>
-    <col min="6" max="6" width="5.44140625" customWidth="1"/>
+    <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="36.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30.5546875" bestFit="1" customWidth="1"/>
@@ -526,6 +526,9 @@
       <c r="E4" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
       <c r="G4" t="s">
         <v>2</v>
       </c>
@@ -545,6 +548,9 @@
       </c>
       <c r="E5">
         <v>125</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
       </c>
       <c r="G5">
         <v>125</v>

</xml_diff>